<commit_message>
added multiple changes to site. added nurses, grid detection, datepicker, etc. trying to implement tkinter GUI to the automator :D
</commit_message>
<xml_diff>
--- a/joborderpersonnels.xlsx
+++ b/joborderpersonnels.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\projects\DTR-Automation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17A41879-825E-4DF0-B6E6-3D9D4E60E378}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{597A7968-971A-44C2-A02D-FE0307E3414D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="14400" windowHeight="15600" xr2:uid="{6831A95B-8140-4EBC-B9A1-5EB659DA3437}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6831A95B-8140-4EBC-B9A1-5EB659DA3437}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,10 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
-  <si>
-    <t>Name</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="12">
   <si>
     <t>ADAYA, JAYNEL</t>
   </si>
@@ -54,6 +51,27 @@
   </si>
   <si>
     <t>ALCALDE, JUDE</t>
+  </si>
+  <si>
+    <t>JobOrderName</t>
+  </si>
+  <si>
+    <t>PONTE, JOSEF</t>
+  </si>
+  <si>
+    <t>NurseName</t>
+  </si>
+  <si>
+    <t>TANSIONGCO, JOHN</t>
+  </si>
+  <si>
+    <t>JURINARIO, NICOLE</t>
+  </si>
+  <si>
+    <t>OLLOSA, JASON</t>
+  </si>
+  <si>
+    <t>TestNames</t>
   </si>
 </sst>
 </file>
@@ -434,40 +452,72 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1210EA2A-C124-48CE-BE32-5813A5795DF8}">
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.28515625" customWidth="1"/>
+    <col min="2" max="2" width="33" customWidth="1"/>
+    <col min="3" max="3" width="17.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>0</v>
       </c>
+      <c r="B2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" t="s">
+        <v>6</v>
+      </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>1</v>
       </c>
+      <c r="B3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" t="s">
+        <v>8</v>
+      </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>2</v>
       </c>
+      <c r="B5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" t="s">
+        <v>10</v>
+      </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
code refactored by claude, testing on monday
</commit_message>
<xml_diff>
--- a/joborderpersonnels.xlsx
+++ b/joborderpersonnels.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\projects\DTR-Automation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CC355CC-2B7B-4DC1-8F22-4C769F889258}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B52D89DA-B3A9-4CB6-961B-CC38BAD287D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="14400" windowHeight="15600" xr2:uid="{6831A95B-8140-4EBC-B9A1-5EB659DA3437}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6831A95B-8140-4EBC-B9A1-5EB659DA3437}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="58">
   <si>
     <t>ADAYA, JAYNEL</t>
   </si>
@@ -80,9 +80,6 @@
     <t>BALTAR, WENDY</t>
   </si>
   <si>
-    <t>BATIDUN, PAUL</t>
-  </si>
-  <si>
     <t>BATOLLO, ARVIE</t>
   </si>
   <si>
@@ -95,18 +92,12 @@
     <t>DELES, MECHEL</t>
   </si>
   <si>
-    <t>DELOVIAR, IZABELE</t>
-  </si>
-  <si>
     <t>DORIN, WENILIE</t>
   </si>
   <si>
     <t>ESPADA, JONEL</t>
   </si>
   <si>
-    <t>ESPAÑOL, EL</t>
-  </si>
-  <si>
     <t>FALALIMPA, ZYRENE</t>
   </si>
   <si>
@@ -164,9 +155,6 @@
     <t>DAILAN, MARJON</t>
   </si>
   <si>
-    <t>DEÑOLA, SERJ</t>
-  </si>
-  <si>
     <t>DENOSTA, CLEARIE</t>
   </si>
   <si>
@@ -210,6 +198,18 @@
   </si>
   <si>
     <t>BANATE, RYJEAN</t>
+  </si>
+  <si>
+    <t>BATIDUAN, PAUL</t>
+  </si>
+  <si>
+    <t>DELOVIAR, IZABELLE</t>
+  </si>
+  <si>
+    <t>SERJ JOSEF</t>
+  </si>
+  <si>
+    <t>EL JUN GALLARDO</t>
   </si>
 </sst>
 </file>
@@ -665,12 +665,12 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -680,192 +680,192 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>14</v>
+        <v>54</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>19</v>
+        <v>55</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>42</v>
+        <v>56</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>22</v>
+        <v>57</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.25">
@@ -875,25 +875,26 @@
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>